<commit_message>
feat: 完成CPU2核心板基础测量与故障框架（CPU2 V0.1.0.0 / CPU3 V0.0.0.1 / 无线主机 V4.1）
版本：
- CPU2：V0.1.0.0（历史提交编号）
- CPU3：V0.0.0.1（历史提交编号）
- 无线主机：V4.1（历史工程目录标识）

协议版本/兼容性：
- 涉及 DSM、LTD 或无线传感器通信；协议口径以该历史提交的代码树为准。

本次修改：
- 形成 CPU2 新称重工程的测量调度、故障管理、传感器、电机和参数存储基础。
- 同步整理早期 CPU3、迷你板及无线主机工程。

验证：
- 提交差异复核：通过；本次仅重写说明，代码树保持不变。
</commit_message>
<xml_diff>
--- a/LTD_MAIN_NEW_WEIGHT/docs/LTD故障代码表.xlsx
+++ b/LTD_MAIN_NEW_WEIGHT/docs/LTD故障代码表.xlsx
@@ -1,13 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12255"/>
+    <workbookView windowWidth="12225" windowHeight="6030"/>
   </bookViews>
   <sheets>
     <sheet name="总表" sheetId="1" r:id="rId1"/>
+    <sheet name="保持寄存器" sheetId="2" r:id="rId2"/>
+    <sheet name="输入寄存器" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -236,7 +238,7 @@
     <t>MEASUREMENT_ZERO_CALIB_TIMEOUT</t>
   </si>
   <si>
-    <t>标定零点超限次</t>
+    <t>标定零点超限</t>
   </si>
   <si>
     <t>MEASUREMENT_OVERSPEED</t>
@@ -1520,6 +1522,7 @@
     <col min="3" max="4" width="12.875" customWidth="1"/>
     <col min="5" max="5" width="38.75" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="8" max="17" width="9" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:17">
@@ -1556,9 +1559,6 @@
     </row>
     <row r="2" spans="4:17">
       <c r="D2" s="1"/>
-      <c r="E2"/>
-      <c r="F2"/>
-      <c r="G2"/>
       <c r="H2">
         <v>1</v>
       </c>
@@ -2319,4 +2319,26 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: 重构CPU2液位流程并整理工程目录（CPU2 V0.4.0.1 / CPU3 V0.5.0.1）
版本：
- CPU2：V0.4.0.1（历史提交编号）
- CPU3：V0.5.0.1（历史提交编号）

协议版本/兼容性：
- 涉及 DSM、LTD 或无线传感器通信；协议口径以该历史提交的代码树为准。

本次修改：
- 重构找液位、液位跟随、称重和传感器处理。
- 移动 CPU2 Core 文件到应用目录，并同步 CPU3 协议映射。

验证：
- 提交差异复核：通过；本次仅重写说明，代码树保持不变。
</commit_message>
<xml_diff>
--- a/LTD_MAIN_NEW_WEIGHT/docs/LTD故障代码表.xlsx
+++ b/LTD_MAIN_NEW_WEIGHT/docs/LTD故障代码表.xlsx
@@ -4,12 +4,12 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="12225" windowHeight="6030"/>
+    <workbookView windowWidth="32565" windowHeight="17655"/>
   </bookViews>
   <sheets>
     <sheet name="总表" sheetId="1" r:id="rId1"/>
-    <sheet name="保持寄存器" sheetId="2" r:id="rId2"/>
-    <sheet name="输入寄存器" sheetId="3" r:id="rId3"/>
+    <sheet name="设备参数" sheetId="4" r:id="rId2"/>
+    <sheet name="测量结果" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="366">
   <si>
     <t>故障类型</t>
   </si>
@@ -368,6 +368,765 @@
   </si>
   <si>
     <t>电源波动异常</t>
+  </si>
+  <si>
+    <t>1. 基础配置参数</t>
+  </si>
+  <si>
+    <t>参数名</t>
+  </si>
+  <si>
+    <t>类型</t>
+  </si>
+  <si>
+    <t>描述</t>
+  </si>
+  <si>
+    <t>备注</t>
+  </si>
+  <si>
+    <t>command</t>
+  </si>
+  <si>
+    <t>CommandType</t>
+  </si>
+  <si>
+    <t>当前指令</t>
+  </si>
+  <si>
+    <t>指令类型</t>
+  </si>
+  <si>
+    <t>tankHeight</t>
+  </si>
+  <si>
+    <t>uint32_t</t>
+  </si>
+  <si>
+    <t>罐高</t>
+  </si>
+  <si>
+    <t>储罐总高度</t>
+  </si>
+  <si>
+    <t>blindZone</t>
+  </si>
+  <si>
+    <t>盲区</t>
+  </si>
+  <si>
+    <t>测量盲区距离</t>
+  </si>
+  <si>
+    <t>waterBlindZone</t>
+  </si>
+  <si>
+    <t>水位盲区</t>
+  </si>
+  <si>
+    <t>水位测量盲区</t>
+  </si>
+  <si>
+    <t>encoder_wheel_circumference_mm</t>
+  </si>
+  <si>
+    <t>编码轮周长</t>
+  </si>
+  <si>
+    <t>编码器参数</t>
+  </si>
+  <si>
+    <t>sensorType</t>
+  </si>
+  <si>
+    <t>传感器类型</t>
+  </si>
+  <si>
+    <t>传感器型号</t>
+  </si>
+  <si>
+    <t>softwareVersion</t>
+  </si>
+  <si>
+    <t>软件版本</t>
+  </si>
+  <si>
+    <t>软件版本号</t>
+  </si>
+  <si>
+    <t>2. 称重参数</t>
+  </si>
+  <si>
+    <t>empty_weight</t>
+  </si>
+  <si>
+    <t>空载重量</t>
+  </si>
+  <si>
+    <t>传感器空载值</t>
+  </si>
+  <si>
+    <t>full_weight</t>
+  </si>
+  <si>
+    <t>满载称重</t>
+  </si>
+  <si>
+    <t>传感器满载值</t>
+  </si>
+  <si>
+    <t>weight_upper_limit_ratio</t>
+  </si>
+  <si>
+    <t>称重检测上限比例</t>
+  </si>
+  <si>
+    <t>超重保护</t>
+  </si>
+  <si>
+    <t>weight_lower_limit_ratio</t>
+  </si>
+  <si>
+    <t>称重检测下限比例</t>
+  </si>
+  <si>
+    <t>欠重保护</t>
+  </si>
+  <si>
+    <t>3. 零点测量参数</t>
+  </si>
+  <si>
+    <t>findZeroDownDistance</t>
+  </si>
+  <si>
+    <t>找零点下行距离</t>
+  </si>
+  <si>
+    <t>零点校准距离</t>
+  </si>
+  <si>
+    <t>4. 密度温度测量参数</t>
+  </si>
+  <si>
+    <t>densityCorrection</t>
+  </si>
+  <si>
+    <t>密度修正值</t>
+  </si>
+  <si>
+    <t>磁通量D</t>
+  </si>
+  <si>
+    <t>temperatureCorrection</t>
+  </si>
+  <si>
+    <t>温度修正值</t>
+  </si>
+  <si>
+    <t>磁通量T</t>
+  </si>
+  <si>
+    <t>5. 测量任务配置</t>
+  </si>
+  <si>
+    <t>requireBottomMeasurement</t>
+  </si>
+  <si>
+    <t>是否需要测量罐底</t>
+  </si>
+  <si>
+    <t>0-否,1-是</t>
+  </si>
+  <si>
+    <t>requireWaterMeasurement</t>
+  </si>
+  <si>
+    <t>是否需要测量水位</t>
+  </si>
+  <si>
+    <t>requireSinglePointDensity</t>
+  </si>
+  <si>
+    <t>是否需要测量单点密度</t>
+  </si>
+  <si>
+    <t>spreadMeasurementOrder</t>
+  </si>
+  <si>
+    <t>分布测量顺序</t>
+  </si>
+  <si>
+    <t>测量顺序</t>
+  </si>
+  <si>
+    <t>spreadMeasurementMode</t>
+  </si>
+  <si>
+    <t>分布测量模式</t>
+  </si>
+  <si>
+    <t>测量模式</t>
+  </si>
+  <si>
+    <t>spreadMeasurementCount</t>
+  </si>
+  <si>
+    <t>分布测量数量</t>
+  </si>
+  <si>
+    <t>测量点数量</t>
+  </si>
+  <si>
+    <t>spreadMeasurementDistance</t>
+  </si>
+  <si>
+    <t>分布测量间距</t>
+  </si>
+  <si>
+    <t>点间距</t>
+  </si>
+  <si>
+    <t>spreadTopLimit</t>
+  </si>
+  <si>
+    <t>分布测量上限（距液面）</t>
+  </si>
+  <si>
+    <t>上限距离</t>
+  </si>
+  <si>
+    <t>spreadBottomLimit</t>
+  </si>
+  <si>
+    <t>分布测量下限（距罐底）</t>
+  </si>
+  <si>
+    <t>下限距离</t>
+  </si>
+  <si>
+    <t>spreadPointHoverTime</t>
+  </si>
+  <si>
+    <t>第一测量点悬停时间</t>
+  </si>
+  <si>
+    <t>悬停时间</t>
+  </si>
+  <si>
+    <t>6. 水位测量参数</t>
+  </si>
+  <si>
+    <t>waterLevelCorrection</t>
+  </si>
+  <si>
+    <t>水位修正值</t>
+  </si>
+  <si>
+    <t>水位校准</t>
+  </si>
+  <si>
+    <t>maxDownDistance</t>
+  </si>
+  <si>
+    <t>水位测量最大下行距离</t>
+  </si>
+  <si>
+    <t>盲区下行距离</t>
+  </si>
+  <si>
+    <t>7. 实高测量参数</t>
+  </si>
+  <si>
+    <t>refreshTankHeightFlag</t>
+  </si>
+  <si>
+    <t>是否更新液位罐高</t>
+  </si>
+  <si>
+    <t>maxTankHeightDeviation</t>
+  </si>
+  <si>
+    <t>罐高最大变化范围</t>
+  </si>
+  <si>
+    <t>允许偏差</t>
+  </si>
+  <si>
+    <t>initialTankHeight</t>
+  </si>
+  <si>
+    <t>初始实高</t>
+  </si>
+  <si>
+    <t>初始罐高</t>
+  </si>
+  <si>
+    <t>currentTankHeight</t>
+  </si>
+  <si>
+    <t>当前实高</t>
+  </si>
+  <si>
+    <t>当前罐高</t>
+  </si>
+  <si>
+    <t>8. 液位测量参数</t>
+  </si>
+  <si>
+    <t>oilLevelThreshold</t>
+  </si>
+  <si>
+    <t>液位跟随阈值</t>
+  </si>
+  <si>
+    <t>液位检测阈值</t>
+  </si>
+  <si>
+    <t>liquidLevelMeasurementMethod</t>
+  </si>
+  <si>
+    <t>液位测量方式</t>
+  </si>
+  <si>
+    <t>测量方法</t>
+  </si>
+  <si>
+    <t>9. 报警输出参数</t>
+  </si>
+  <si>
+    <t>AlarmHighDO</t>
+  </si>
+  <si>
+    <t>高液位报警输出</t>
+  </si>
+  <si>
+    <t>数字输出</t>
+  </si>
+  <si>
+    <t>AlarmLowDO</t>
+  </si>
+  <si>
+    <t>低液位报警输出</t>
+  </si>
+  <si>
+    <t>10. 4-20mA模拟输出参数</t>
+  </si>
+  <si>
+    <t>CurrentRangeStart_mA</t>
+  </si>
+  <si>
+    <t>电流量程起始值</t>
+  </si>
+  <si>
+    <t>4mA对应值</t>
+  </si>
+  <si>
+    <t>CurrentRangeEnd_mA</t>
+  </si>
+  <si>
+    <t>电流量程结束值</t>
+  </si>
+  <si>
+    <t>20mA对应值</t>
+  </si>
+  <si>
+    <t>AlarmHighAO</t>
+  </si>
+  <si>
+    <t>模拟输出</t>
+  </si>
+  <si>
+    <t>AlarmLowAO</t>
+  </si>
+  <si>
+    <t>InitialCurrent_mA</t>
+  </si>
+  <si>
+    <t>初始化电流值</t>
+  </si>
+  <si>
+    <t>初始电流</t>
+  </si>
+  <si>
+    <t>AOHighCurrent_mA</t>
+  </si>
+  <si>
+    <t>AO高报电流值</t>
+  </si>
+  <si>
+    <t>高报警电流</t>
+  </si>
+  <si>
+    <t>AOLowCurrent_mA</t>
+  </si>
+  <si>
+    <t>AO低报电流值</t>
+  </si>
+  <si>
+    <t>低报警电流</t>
+  </si>
+  <si>
+    <t>FaultCurrent_mA</t>
+  </si>
+  <si>
+    <t>故障模式电流值</t>
+  </si>
+  <si>
+    <t>故障电流</t>
+  </si>
+  <si>
+    <t>DebugCurrent_mA</t>
+  </si>
+  <si>
+    <t>调试模式电流值</t>
+  </si>
+  <si>
+    <t>调试电流</t>
+  </si>
+  <si>
+    <t>11. 校验参数</t>
+  </si>
+  <si>
+    <t>crc</t>
+  </si>
+  <si>
+    <t>CRC校验字段</t>
+  </si>
+  <si>
+    <t>数据校验</t>
+  </si>
+  <si>
+    <t>结构体</t>
+  </si>
+  <si>
+    <t>字段名</t>
+  </si>
+  <si>
+    <t>数据类型</t>
+  </si>
+  <si>
+    <t>说明</t>
+  </si>
+  <si>
+    <t>DeviceStatus</t>
+  </si>
+  <si>
+    <t>work_mode</t>
+  </si>
+  <si>
+    <t>工作模式（0:工作模式 1:调试模式 78:解锁模式）</t>
+  </si>
+  <si>
+    <t>device_state</t>
+  </si>
+  <si>
+    <t>DeviceState</t>
+  </si>
+  <si>
+    <t>设备运行状态</t>
+  </si>
+  <si>
+    <t>error_code</t>
+  </si>
+  <si>
+    <t>当前错误码（0表示无错误）</t>
+  </si>
+  <si>
+    <t>current_command</t>
+  </si>
+  <si>
+    <t>zero_point_status</t>
+  </si>
+  <si>
+    <t>uint8_t</t>
+  </si>
+  <si>
+    <t>零点状态（0-正常 1-需要回零）</t>
+  </si>
+  <si>
+    <t>DensityMeasurement</t>
+  </si>
+  <si>
+    <t>temperature</t>
+  </si>
+  <si>
+    <t>温度</t>
+  </si>
+  <si>
+    <t>density</t>
+  </si>
+  <si>
+    <t>密度</t>
+  </si>
+  <si>
+    <t>temperature_position</t>
+  </si>
+  <si>
+    <t>温度密度位置</t>
+  </si>
+  <si>
+    <t>standard_density</t>
+  </si>
+  <si>
+    <t>标准密度</t>
+  </si>
+  <si>
+    <t>vcf20</t>
+  </si>
+  <si>
+    <t>体积修正系数 (VCF20)</t>
+  </si>
+  <si>
+    <t>weight_density</t>
+  </si>
+  <si>
+    <t>计重密度</t>
+  </si>
+  <si>
+    <t>DensityDistribution</t>
+  </si>
+  <si>
+    <t>average_temperature</t>
+  </si>
+  <si>
+    <t>平均温度</t>
+  </si>
+  <si>
+    <t>average_density</t>
+  </si>
+  <si>
+    <t>平均密度</t>
+  </si>
+  <si>
+    <t>average_standard_density</t>
+  </si>
+  <si>
+    <t>平均标准密度</t>
+  </si>
+  <si>
+    <t>average_vcf20</t>
+  </si>
+  <si>
+    <t>平均体积修正系数 (VCF20)</t>
+  </si>
+  <si>
+    <t>average_weight_density</t>
+  </si>
+  <si>
+    <t>平均计重密度</t>
+  </si>
+  <si>
+    <t>measurement_points</t>
+  </si>
+  <si>
+    <t>实际测量点数</t>
+  </si>
+  <si>
+    <t>Density_oil_level</t>
+  </si>
+  <si>
+    <t>密度分布测量时的液位值</t>
+  </si>
+  <si>
+    <t>single_density_data</t>
+  </si>
+  <si>
+    <t>DensityMeasurement[100]</t>
+  </si>
+  <si>
+    <t>100个点的密度测量数据</t>
+  </si>
+  <si>
+    <t>ZeroCalibration</t>
+  </si>
+  <si>
+    <t>zero_encoder_turns</t>
+  </si>
+  <si>
+    <t>零点编码器圈数</t>
+  </si>
+  <si>
+    <t>zero_encoder_value</t>
+  </si>
+  <si>
+    <t>零点编码器编码值</t>
+  </si>
+  <si>
+    <t>DebugData</t>
+  </si>
+  <si>
+    <t>current_encoder_value</t>
+  </si>
+  <si>
+    <t>int32_t</t>
+  </si>
+  <si>
+    <t>当前编码值</t>
+  </si>
+  <si>
+    <t>sensor_position</t>
+  </si>
+  <si>
+    <t>传感器位置</t>
+  </si>
+  <si>
+    <t>cable_length</t>
+  </si>
+  <si>
+    <t>尺带长度</t>
+  </si>
+  <si>
+    <t>frequency</t>
+  </si>
+  <si>
+    <t>频率</t>
+  </si>
+  <si>
+    <t>温度 (单位:0.01°C)</t>
+  </si>
+  <si>
+    <t>air_frequency</t>
+  </si>
+  <si>
+    <t>空气中频率</t>
+  </si>
+  <si>
+    <t>current_amplitude</t>
+  </si>
+  <si>
+    <t>当前幅值</t>
+  </si>
+  <si>
+    <t>water_level_voltage</t>
+  </si>
+  <si>
+    <t>水位电压值/电容值</t>
+  </si>
+  <si>
+    <t>ActualHeightMeasurement</t>
+  </si>
+  <si>
+    <t>calibrated_liquid_level</t>
+  </si>
+  <si>
+    <t>标定液位时实高</t>
+  </si>
+  <si>
+    <t>current_real_height</t>
+  </si>
+  <si>
+    <t>OilMeasurement</t>
+  </si>
+  <si>
+    <t>oil_level</t>
+  </si>
+  <si>
+    <t>液位跟随液位值</t>
+  </si>
+  <si>
+    <t>oil_frequency</t>
+  </si>
+  <si>
+    <t>油中频率</t>
+  </si>
+  <si>
+    <t>follow_frequency</t>
+  </si>
+  <si>
+    <t>液位跟随频率</t>
+  </si>
+  <si>
+    <t>current_frequency</t>
+  </si>
+  <si>
+    <t>当前频率</t>
+  </si>
+  <si>
+    <t>WaterMeasurement</t>
+  </si>
+  <si>
+    <t>water_level</t>
+  </si>
+  <si>
+    <t>测量水位的值</t>
+  </si>
+  <si>
+    <t>zero_capacitance</t>
+  </si>
+  <si>
+    <t>float</t>
+  </si>
+  <si>
+    <t>零点电容</t>
+  </si>
+  <si>
+    <t>oil_capacitance</t>
+  </si>
+  <si>
+    <t>油中电容</t>
+  </si>
+  <si>
+    <t>current_capacitance</t>
+  </si>
+  <si>
+    <t>当前电容</t>
+  </si>
+  <si>
+    <t>MeasurementResult</t>
+  </si>
+  <si>
+    <t>device_status</t>
+  </si>
+  <si>
+    <t>设备状态</t>
+  </si>
+  <si>
+    <t>oil_measurement</t>
+  </si>
+  <si>
+    <t>液位测量数据</t>
+  </si>
+  <si>
+    <t>water_measurement</t>
+  </si>
+  <si>
+    <t>水位测量数据</t>
+  </si>
+  <si>
+    <t>zero_calibration</t>
+  </si>
+  <si>
+    <t>标定零点数据</t>
+  </si>
+  <si>
+    <t>height_measurement</t>
+  </si>
+  <si>
+    <t>实高测量数据</t>
+  </si>
+  <si>
+    <t>debug_data</t>
+  </si>
+  <si>
+    <t>调试数据</t>
+  </si>
+  <si>
+    <t>single_point_measurement</t>
+  </si>
+  <si>
+    <t>单点测量数据</t>
+  </si>
+  <si>
+    <t>single_point_monitoring</t>
+  </si>
+  <si>
+    <t>单点监测数据</t>
+  </si>
+  <si>
+    <t>density_distribution</t>
+  </si>
+  <si>
+    <t>密度分布测量数据</t>
   </si>
 </sst>
 </file>
@@ -380,9 +1139,48 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="25">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14.05"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.5"/>
+      <color rgb="FF000000"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <color rgb="FF000000"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -727,12 +1525,42 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="11">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFE0E0E0"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFE0E0E0"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFE0E0E0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFE0E0E0"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -853,139 +1681,158 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1526,39 +2373,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:17">
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="8"/>
+      <c r="P1" s="8"/>
+      <c r="Q1" s="8"/>
     </row>
     <row r="2" spans="4:17">
-      <c r="D2" s="1"/>
+      <c r="D2" s="8"/>
       <c r="H2">
         <v>1</v>
       </c>
@@ -1591,13 +2438,13 @@
       </c>
     </row>
     <row r="3" spans="2:6">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="8">
         <v>11</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="8">
         <v>1</v>
       </c>
       <c r="E3" t="s">
@@ -1608,9 +2455,9 @@
       </c>
     </row>
     <row r="4" spans="2:6">
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1">
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8">
         <v>2</v>
       </c>
       <c r="E4" t="s">
@@ -1621,9 +2468,9 @@
       </c>
     </row>
     <row r="5" spans="2:6">
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1">
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8">
         <v>3</v>
       </c>
       <c r="E5" t="s">
@@ -1634,9 +2481,9 @@
       </c>
     </row>
     <row r="6" spans="2:6">
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1">
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8">
         <v>4</v>
       </c>
       <c r="E6" t="s">
@@ -1647,9 +2494,9 @@
       </c>
     </row>
     <row r="7" spans="2:6">
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1">
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8">
         <v>5</v>
       </c>
       <c r="E7" t="s">
@@ -1660,9 +2507,9 @@
       </c>
     </row>
     <row r="8" spans="2:6">
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1">
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8">
         <v>6</v>
       </c>
       <c r="E8" t="s">
@@ -1673,9 +2520,9 @@
       </c>
     </row>
     <row r="9" spans="2:6">
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1">
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8">
         <v>7</v>
       </c>
       <c r="E9" t="s">
@@ -1686,9 +2533,9 @@
       </c>
     </row>
     <row r="10" spans="2:6">
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1">
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8">
         <v>8</v>
       </c>
       <c r="E10" t="s">
@@ -1699,13 +2546,13 @@
       </c>
     </row>
     <row r="11" spans="2:6">
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="8">
         <v>12</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11" s="8">
         <v>1</v>
       </c>
       <c r="E11" t="s">
@@ -1716,9 +2563,9 @@
       </c>
     </row>
     <row r="12" spans="2:6">
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1">
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8">
         <v>2</v>
       </c>
       <c r="E12" t="s">
@@ -1729,9 +2576,9 @@
       </c>
     </row>
     <row r="13" spans="2:6">
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1">
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8">
         <v>3</v>
       </c>
       <c r="E13" t="s">
@@ -1742,9 +2589,9 @@
       </c>
     </row>
     <row r="14" spans="2:6">
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1">
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8">
         <v>4</v>
       </c>
       <c r="E14" t="s">
@@ -1755,9 +2602,9 @@
       </c>
     </row>
     <row r="15" spans="2:6">
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1">
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8">
         <v>5</v>
       </c>
       <c r="E15" t="s">
@@ -1768,9 +2615,9 @@
       </c>
     </row>
     <row r="16" spans="2:6">
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1">
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8">
         <v>6</v>
       </c>
       <c r="E16" t="s">
@@ -1781,9 +2628,9 @@
       </c>
     </row>
     <row r="17" spans="2:6">
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1">
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8">
         <v>7</v>
       </c>
       <c r="E17" t="s">
@@ -1794,9 +2641,9 @@
       </c>
     </row>
     <row r="18" spans="2:6">
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1">
+      <c r="B18" s="8"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8">
         <v>8</v>
       </c>
       <c r="E18" t="s">
@@ -1807,13 +2654,13 @@
       </c>
     </row>
     <row r="19" spans="2:6">
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="1">
+      <c r="C19" s="8">
         <v>13</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="8">
         <v>1</v>
       </c>
       <c r="E19" t="s">
@@ -1824,9 +2671,9 @@
       </c>
     </row>
     <row r="20" spans="2:6">
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1">
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8">
         <v>2</v>
       </c>
       <c r="E20" t="s">
@@ -1837,9 +2684,9 @@
       </c>
     </row>
     <row r="21" spans="2:6">
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1">
+      <c r="B21" s="8"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8">
         <v>3</v>
       </c>
       <c r="E21" t="s">
@@ -1850,9 +2697,9 @@
       </c>
     </row>
     <row r="22" spans="2:6">
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1">
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8">
         <v>4</v>
       </c>
       <c r="E22" t="s">
@@ -1863,9 +2710,9 @@
       </c>
     </row>
     <row r="23" spans="2:6">
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1">
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8">
         <v>5</v>
       </c>
       <c r="E23" t="s">
@@ -1876,9 +2723,9 @@
       </c>
     </row>
     <row r="24" spans="2:6">
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1">
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8">
         <v>6</v>
       </c>
       <c r="E24" t="s">
@@ -1889,13 +2736,13 @@
       </c>
     </row>
     <row r="25" spans="2:6">
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C25" s="1">
+      <c r="C25" s="8">
         <v>14</v>
       </c>
-      <c r="D25" s="1">
+      <c r="D25" s="8">
         <v>1</v>
       </c>
       <c r="E25" t="s">
@@ -1906,9 +2753,9 @@
       </c>
     </row>
     <row r="26" spans="2:6">
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1">
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8">
         <v>2</v>
       </c>
       <c r="E26" t="s">
@@ -1919,9 +2766,9 @@
       </c>
     </row>
     <row r="27" spans="2:6">
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1">
+      <c r="B27" s="8"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8">
         <v>3</v>
       </c>
       <c r="E27" t="s">
@@ -1932,9 +2779,9 @@
       </c>
     </row>
     <row r="28" spans="2:6">
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1">
+      <c r="B28" s="8"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8">
         <v>4</v>
       </c>
       <c r="E28" t="s">
@@ -1945,9 +2792,9 @@
       </c>
     </row>
     <row r="29" spans="2:6">
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1">
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8">
         <v>5</v>
       </c>
       <c r="E29" t="s">
@@ -1958,13 +2805,13 @@
       </c>
     </row>
     <row r="30" spans="2:6">
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C30" s="1">
+      <c r="C30" s="8">
         <v>15</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="8">
         <v>1</v>
       </c>
       <c r="E30" t="s">
@@ -1975,9 +2822,9 @@
       </c>
     </row>
     <row r="31" spans="2:6">
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1">
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8">
         <v>2</v>
       </c>
       <c r="E31" t="s">
@@ -1988,9 +2835,9 @@
       </c>
     </row>
     <row r="32" spans="2:6">
-      <c r="B32" s="1"/>
-      <c r="C32" s="1"/>
-      <c r="D32" s="1">
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8">
         <v>3</v>
       </c>
       <c r="E32" t="s">
@@ -2001,9 +2848,9 @@
       </c>
     </row>
     <row r="33" spans="2:6">
-      <c r="B33" s="1"/>
-      <c r="C33" s="1"/>
-      <c r="D33" s="1">
+      <c r="B33" s="8"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8">
         <v>4</v>
       </c>
       <c r="E33" t="s">
@@ -2014,9 +2861,9 @@
       </c>
     </row>
     <row r="34" spans="2:6">
-      <c r="B34" s="1"/>
-      <c r="C34" s="1"/>
-      <c r="D34" s="1">
+      <c r="B34" s="8"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8">
         <v>5</v>
       </c>
       <c r="E34" t="s">
@@ -2027,9 +2874,9 @@
       </c>
     </row>
     <row r="35" spans="2:6">
-      <c r="B35" s="1"/>
-      <c r="C35" s="1"/>
-      <c r="D35" s="1">
+      <c r="B35" s="8"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8">
         <v>6</v>
       </c>
       <c r="E35" t="s">
@@ -2040,9 +2887,9 @@
       </c>
     </row>
     <row r="36" spans="2:6">
-      <c r="B36" s="1"/>
-      <c r="C36" s="1"/>
-      <c r="D36" s="1">
+      <c r="B36" s="8"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8">
         <v>7</v>
       </c>
       <c r="E36" t="s">
@@ -2053,9 +2900,9 @@
       </c>
     </row>
     <row r="37" spans="2:6">
-      <c r="B37" s="1"/>
-      <c r="C37" s="1"/>
-      <c r="D37" s="1">
+      <c r="B37" s="8"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8">
         <v>8</v>
       </c>
       <c r="E37" t="s">
@@ -2066,9 +2913,9 @@
       </c>
     </row>
     <row r="38" spans="2:6">
-      <c r="B38" s="1"/>
-      <c r="C38" s="1"/>
-      <c r="D38" s="1">
+      <c r="B38" s="8"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8">
         <v>9</v>
       </c>
       <c r="E38" t="s">
@@ -2079,9 +2926,9 @@
       </c>
     </row>
     <row r="39" spans="2:6">
-      <c r="B39" s="1"/>
-      <c r="C39" s="1"/>
-      <c r="D39" s="1">
+      <c r="B39" s="8"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8">
         <v>10</v>
       </c>
       <c r="E39" t="s">
@@ -2092,9 +2939,9 @@
       </c>
     </row>
     <row r="40" spans="2:6">
-      <c r="B40" s="1"/>
-      <c r="C40" s="1"/>
-      <c r="D40" s="1">
+      <c r="B40" s="8"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8">
         <v>11</v>
       </c>
       <c r="E40" t="s">
@@ -2105,13 +2952,13 @@
       </c>
     </row>
     <row r="41" spans="2:6">
-      <c r="B41" s="1" t="s">
+      <c r="B41" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="C41" s="1">
+      <c r="C41" s="8">
         <v>16</v>
       </c>
-      <c r="D41" s="1">
+      <c r="D41" s="8">
         <v>1</v>
       </c>
       <c r="E41" t="s">
@@ -2122,9 +2969,9 @@
       </c>
     </row>
     <row r="42" spans="2:6">
-      <c r="B42" s="1"/>
-      <c r="C42" s="1"/>
-      <c r="D42" s="1">
+      <c r="B42" s="8"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8">
         <v>2</v>
       </c>
       <c r="E42" t="s">
@@ -2135,9 +2982,9 @@
       </c>
     </row>
     <row r="43" spans="2:6">
-      <c r="B43" s="1"/>
-      <c r="C43" s="1"/>
-      <c r="D43" s="1">
+      <c r="B43" s="8"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="8">
         <v>3</v>
       </c>
       <c r="E43" t="s">
@@ -2148,9 +2995,9 @@
       </c>
     </row>
     <row r="44" spans="2:6">
-      <c r="B44" s="1"/>
-      <c r="C44" s="1"/>
-      <c r="D44" s="1">
+      <c r="B44" s="8"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8">
         <v>4</v>
       </c>
       <c r="E44" t="s">
@@ -2161,13 +3008,13 @@
       </c>
     </row>
     <row r="45" spans="2:6">
-      <c r="B45" s="1" t="s">
+      <c r="B45" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="C45" s="1">
+      <c r="C45" s="8">
         <v>17</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="8">
         <v>1</v>
       </c>
       <c r="E45" t="s">
@@ -2178,9 +3025,9 @@
       </c>
     </row>
     <row r="46" spans="2:6">
-      <c r="B46" s="1"/>
-      <c r="C46" s="1"/>
-      <c r="D46" s="1">
+      <c r="B46" s="8"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="8">
         <v>2</v>
       </c>
       <c r="E46" t="s">
@@ -2191,9 +3038,9 @@
       </c>
     </row>
     <row r="47" spans="2:6">
-      <c r="B47" s="1"/>
-      <c r="C47" s="1"/>
-      <c r="D47" s="1">
+      <c r="B47" s="8"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="8">
         <v>3</v>
       </c>
       <c r="E47" t="s">
@@ -2204,9 +3051,9 @@
       </c>
     </row>
     <row r="48" spans="2:6">
-      <c r="B48" s="1"/>
-      <c r="C48" s="1"/>
-      <c r="D48" s="1">
+      <c r="B48" s="8"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8">
         <v>4</v>
       </c>
       <c r="E48" t="s">
@@ -2217,9 +3064,9 @@
       </c>
     </row>
     <row r="49" spans="2:6">
-      <c r="B49" s="1"/>
-      <c r="C49" s="1"/>
-      <c r="D49" s="1">
+      <c r="B49" s="8"/>
+      <c r="C49" s="8"/>
+      <c r="D49" s="8">
         <v>5</v>
       </c>
       <c r="E49" t="s">
@@ -2230,13 +3077,13 @@
       </c>
     </row>
     <row r="50" spans="2:6">
-      <c r="B50" s="1" t="s">
+      <c r="B50" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="C50" s="1">
+      <c r="C50" s="8">
         <v>18</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="8">
         <v>1</v>
       </c>
       <c r="E50" t="s">
@@ -2247,9 +3094,9 @@
       </c>
     </row>
     <row r="51" spans="2:6">
-      <c r="B51" s="1"/>
-      <c r="C51" s="1"/>
-      <c r="D51" s="1">
+      <c r="B51" s="8"/>
+      <c r="C51" s="8"/>
+      <c r="D51" s="8">
         <v>2</v>
       </c>
       <c r="E51" t="s">
@@ -2260,9 +3107,9 @@
       </c>
     </row>
     <row r="52" spans="2:6">
-      <c r="B52" s="1"/>
-      <c r="C52" s="1"/>
-      <c r="D52" s="1">
+      <c r="B52" s="8"/>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8">
         <v>3</v>
       </c>
       <c r="E52" t="s">
@@ -2273,16 +3120,16 @@
       </c>
     </row>
     <row r="53" spans="4:4">
-      <c r="D53" s="1"/>
+      <c r="D53" s="8"/>
     </row>
     <row r="54" spans="4:4">
-      <c r="D54" s="1"/>
+      <c r="D54" s="8"/>
     </row>
     <row r="55" spans="4:4">
-      <c r="D55" s="1"/>
+      <c r="D55" s="8"/>
     </row>
     <row r="56" spans="4:4">
-      <c r="D56" s="1"/>
+      <c r="D56" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="23">
@@ -2324,9 +3171,873 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
-  <sheetData/>
+  <dimension ref="A2:D105"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="3"/>
+  <cols>
+    <col min="1" max="1" width="23.875" customWidth="1"/>
+    <col min="2" max="2" width="18.625" customWidth="1"/>
+    <col min="3" max="3" width="19.75" customWidth="1"/>
+    <col min="4" max="4" width="35.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="18.75" spans="1:1">
+      <c r="A2" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="3" ht="14.25"/>
+    <row r="4" ht="14.25" spans="1:4">
+      <c r="A4" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" ht="14.25" spans="1:4">
+      <c r="A5" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="6" ht="14.25" spans="1:4">
+      <c r="A6" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="7" ht="14.25" spans="1:4">
+      <c r="A7" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="8" ht="14.25" spans="1:4">
+      <c r="A8" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="9" ht="26.25" spans="1:4">
+      <c r="A9" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="10" ht="14.25" spans="1:4">
+      <c r="A10" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="11" ht="14.25" spans="1:4">
+      <c r="A11" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="13" ht="18.75" spans="1:1">
+      <c r="A13" s="3" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="14" ht="14.25"/>
+    <row r="15" ht="14.25" spans="1:4">
+      <c r="A15" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="16" ht="14.25" spans="1:4">
+      <c r="A16" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="17" ht="14.25" spans="1:4">
+      <c r="A17" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="18" ht="14.25" spans="1:4">
+      <c r="A18" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="19" ht="14.25" spans="1:4">
+      <c r="A19" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="21" ht="18.75" spans="1:1">
+      <c r="A21" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="22" ht="14.25"/>
+    <row r="23" ht="14.25" spans="1:4">
+      <c r="A23" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="24" ht="14.25" spans="1:4">
+      <c r="A24" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="26" ht="18.75" spans="1:1">
+      <c r="A26" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="27" ht="14.25"/>
+    <row r="28" ht="14.25" spans="1:4">
+      <c r="A28" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="29" ht="14.25" spans="1:4">
+      <c r="A29" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="30" ht="14.25" spans="1:4">
+      <c r="A30" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="32" ht="18.75" spans="1:1">
+      <c r="A32" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="33" ht="14.25"/>
+    <row r="34" ht="14.25" spans="1:4">
+      <c r="A34" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="35" ht="14.25" spans="1:4">
+      <c r="A35" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="36" ht="14.25" spans="1:4">
+      <c r="A36" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="37" ht="14.25" spans="1:4">
+      <c r="A37" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="38" ht="14.25" spans="1:4">
+      <c r="A38" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="39" ht="14.25" spans="1:4">
+      <c r="A39" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="40" ht="14.25" spans="1:4">
+      <c r="A40" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="41" ht="14.25" spans="1:4">
+      <c r="A41" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="42" ht="26.25" spans="1:4">
+      <c r="A42" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="43" ht="26.25" spans="1:4">
+      <c r="A43" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="44" ht="14.25" spans="1:4">
+      <c r="A44" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="46" ht="18.75" spans="1:1">
+      <c r="A46" s="3" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="47" ht="14.25"/>
+    <row r="48" ht="14.25" spans="1:4">
+      <c r="A48" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="49" ht="14.25" spans="1:4">
+      <c r="A49" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="50" ht="14.25" spans="1:4">
+      <c r="A50" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="52" ht="18.75" spans="1:1">
+      <c r="A52" s="3" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="53" ht="14.25"/>
+    <row r="54" ht="14.25" spans="1:4">
+      <c r="A54" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="55" ht="14.25" spans="1:4">
+      <c r="A55" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B55" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C55" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="56" ht="14.25" spans="1:4">
+      <c r="A56" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="57" ht="14.25" spans="1:4">
+      <c r="A57" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C57" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="58" ht="14.25" spans="1:4">
+      <c r="A58" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="60" ht="18.75" spans="1:1">
+      <c r="A60" s="3" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="61" ht="14.25"/>
+    <row r="62" ht="14.25" spans="1:4">
+      <c r="A62" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="63" ht="14.25" spans="1:4">
+      <c r="A63" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="B63" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C63" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D63" s="5" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="64" ht="26.25" spans="1:4">
+      <c r="A64" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="B64" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="D64" s="5" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="66" ht="18.75" spans="1:1">
+      <c r="A66" s="3" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="67" ht="14.25"/>
+    <row r="68" ht="14.25" spans="1:4">
+      <c r="A68" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="69" ht="14.25" spans="1:4">
+      <c r="A69" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="B69" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C69" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="D69" s="5" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="70" ht="14.25" spans="1:4">
+      <c r="A70" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="B70" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C70" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="D70" s="5" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="72" ht="18.75" spans="1:1">
+      <c r="A72" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="73" ht="14.25"/>
+    <row r="74" ht="14.25" spans="1:4">
+      <c r="A74" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="75" ht="14.25" spans="1:4">
+      <c r="A75" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="B75" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C75" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="76" ht="14.25" spans="1:4">
+      <c r="A76" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="B76" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C76" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="D76" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="77" ht="14.25" spans="1:4">
+      <c r="A77" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="B77" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C77" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="D77" s="5" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="78" ht="14.25" spans="1:4">
+      <c r="A78" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="B78" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C78" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="D78" s="5" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="79" ht="14.25" spans="1:4">
+      <c r="A79" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="B79" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C79" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="D79" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="80" ht="14.25" spans="1:4">
+      <c r="A80" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="B80" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C80" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="D80" s="5" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="81" ht="14.25" spans="1:4">
+      <c r="A81" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="B81" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C81" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="D81" s="5" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="82" ht="14.25" spans="1:4">
+      <c r="A82" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="B82" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C82" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D82" s="5" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="83" ht="14.25" spans="1:4">
+      <c r="A83" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="B83" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C83" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="D83" s="5" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="85" ht="18.75" spans="1:1">
+      <c r="A85" s="3" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="86" ht="14.25"/>
+    <row r="87" ht="14.25" spans="1:4">
+      <c r="A87" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="88" ht="14.25" spans="1:4">
+      <c r="A88" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="B88" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C88" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="D88" s="5" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="90" ht="22.5" spans="1:1">
+      <c r="A90" s="6"/>
+    </row>
+    <row r="95" spans="1:1">
+      <c r="A95" s="7"/>
+    </row>
+    <row r="97" spans="1:1">
+      <c r="A97" s="7"/>
+    </row>
+    <row r="99" spans="1:1">
+      <c r="A99" s="7"/>
+    </row>
+    <row r="101" spans="1:1">
+      <c r="A101" s="7"/>
+    </row>
+    <row r="103" spans="1:1">
+      <c r="A103" s="7"/>
+    </row>
+    <row r="105" spans="1:1">
+      <c r="A105" s="7"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
@@ -2335,9 +4046,717 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
-  <sheetData/>
+  <dimension ref="A1:D50"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="3"/>
+  <cols>
+    <col min="1" max="1" width="26" style="1" customWidth="1"/>
+    <col min="2" max="2" width="27.125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="26" style="1" customWidth="1"/>
+    <col min="4" max="4" width="47.875" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="9" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="1" customFormat="1" spans="1:4">
+      <c r="A1" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="2" s="1" customFormat="1" spans="1:4">
+      <c r="A2" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="3" s="1" customFormat="1" spans="1:4">
+      <c r="A3" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="4" s="1" customFormat="1" spans="1:4">
+      <c r="A4" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="5" s="1" customFormat="1" spans="1:4">
+      <c r="A5" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" s="1" customFormat="1" spans="1:4">
+      <c r="A6" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="7" s="1" customFormat="1" spans="1:4">
+      <c r="A7" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="8" s="1" customFormat="1" spans="1:4">
+      <c r="A8" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="9" s="1" customFormat="1" spans="1:4">
+      <c r="A9" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="10" s="1" customFormat="1" spans="1:4">
+      <c r="A10" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="11" s="1" customFormat="1" spans="1:4">
+      <c r="A11" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="12" s="1" customFormat="1" spans="1:4">
+      <c r="A12" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="13" s="1" customFormat="1" spans="1:4">
+      <c r="A13" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="14" s="1" customFormat="1" spans="1:4">
+      <c r="A14" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="15" s="1" customFormat="1" spans="1:4">
+      <c r="A15" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="16" s="1" customFormat="1" spans="1:4">
+      <c r="A16" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="17" s="1" customFormat="1" spans="1:4">
+      <c r="A17" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="18" s="1" customFormat="1" spans="1:4">
+      <c r="A18" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="19" s="1" customFormat="1" spans="1:4">
+      <c r="A19" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="20" s="1" customFormat="1" spans="1:4">
+      <c r="A20" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="21" s="1" customFormat="1" spans="1:4">
+      <c r="A21" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="22" s="1" customFormat="1" spans="1:4">
+      <c r="A22" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="23" s="1" customFormat="1" spans="1:4">
+      <c r="A23" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="24" s="1" customFormat="1" spans="1:4">
+      <c r="A24" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="25" s="1" customFormat="1" spans="1:4">
+      <c r="A25" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="26" s="1" customFormat="1" spans="1:4">
+      <c r="A26" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="27" s="1" customFormat="1" spans="1:4">
+      <c r="A27" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="28" s="1" customFormat="1" spans="1:4">
+      <c r="A28" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="29" s="1" customFormat="1" spans="1:4">
+      <c r="A29" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="30" s="1" customFormat="1" spans="1:4">
+      <c r="A30" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="31" s="1" customFormat="1" spans="1:4">
+      <c r="A31" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="32" s="1" customFormat="1" spans="1:4">
+      <c r="A32" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="33" s="1" customFormat="1" spans="1:4">
+      <c r="A33" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="34" s="1" customFormat="1" spans="1:4">
+      <c r="A34" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="35" s="1" customFormat="1" spans="1:4">
+      <c r="A35" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="36" s="1" customFormat="1" spans="1:4">
+      <c r="A36" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="37" s="1" customFormat="1" spans="1:4">
+      <c r="A37" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="38" s="1" customFormat="1" spans="1:4">
+      <c r="A38" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="39" s="1" customFormat="1" spans="1:4">
+      <c r="A39" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="40" s="1" customFormat="1" spans="1:4">
+      <c r="A40" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="41" s="1" customFormat="1" spans="1:4">
+      <c r="A41" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="42" s="1" customFormat="1" spans="1:4">
+      <c r="A42" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="43" s="1" customFormat="1" spans="1:4">
+      <c r="A43" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="44" s="1" customFormat="1" spans="1:4">
+      <c r="A44" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="45" s="1" customFormat="1" spans="1:4">
+      <c r="A45" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="46" s="1" customFormat="1" spans="1:4">
+      <c r="A46" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="47" s="1" customFormat="1" spans="1:4">
+      <c r="A47" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="48" s="1" customFormat="1" spans="1:4">
+      <c r="A48" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="49" s="1" customFormat="1" spans="1:4">
+      <c r="A49" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="50" s="1" customFormat="1" spans="1:4">
+      <c r="A50" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>365</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>